<commit_message>
qa: registrar visto bueno y criterios DoD aprobados para HU-17 y HU-18
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -823,7 +823,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
@@ -870,7 +869,6 @@
         <v/>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="28" customHeight="1" s="18">
       <c r="A7" s="4" t="inlineStr">
         <is>
@@ -1022,10 +1020,14 @@
       </c>
       <c r="H9" s="10" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="I9" s="14" t="n"/>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="I9" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
       <c r="J9" s="15" t="inlineStr">
         <is>
           <t>CA1. Cada historia tiene su categoría MoSCoW.
@@ -2725,10 +2727,14 @@
       </c>
       <c r="G5" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H5" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H5" s="15" t="inlineStr">
+        <is>
+          <t>Radar del filtro de idoneidad presentado con promedio 3,2 (zona ágil). Referencias a PMI y Agile Alliance.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="32" customHeight="1" s="18">
       <c r="A6" s="16" t="inlineStr">
@@ -2763,10 +2769,14 @@
       </c>
       <c r="G6" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H6" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="inlineStr">
+        <is>
+          <t>Enfoque predictivo vs ágil justificado para cada entregable con modelo de incertidumbre de Stacey.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="32" customHeight="1" s="18">
       <c r="A7" s="16" t="inlineStr">
@@ -2801,10 +2811,14 @@
       </c>
       <c r="G7" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H7" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H7" s="15" t="inlineStr">
+        <is>
+          <t>Explicada combinación simultánea con marco predictivo de gobierno y sprints Scrum.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="32" customHeight="1" s="18">
       <c r="A8" s="16" t="inlineStr">
@@ -2839,10 +2853,14 @@
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H8" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H8" s="15" t="inlineStr">
+        <is>
+          <t>Documento HU-17_Modelo_Hibrido.docx subido y versionado en la carpeta Docs.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="32" customHeight="1" s="18">
       <c r="A9" s="16" t="inlineStr">
@@ -2877,10 +2895,14 @@
       </c>
       <c r="G9" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H9" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H9" s="15" t="inlineStr">
+        <is>
+          <t>Clasificación MoSCoW completa para todos los entregables de la segunda entrega (24p Must, 17p Should, 5p Could, 0p Won't).</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="32" customHeight="1" s="18">
       <c r="A10" s="16" t="inlineStr">
@@ -2915,10 +2937,14 @@
       </c>
       <c r="G10" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H10" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>Must representa exactamente el 52 % del esfuerzo total, cumpliendo la regla de estar por debajo del 60 %.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="32" customHeight="1" s="18">
       <c r="A11" s="16" t="inlineStr">
@@ -2953,10 +2979,14 @@
       </c>
       <c r="G11" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H11" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H11" s="15" t="inlineStr">
+        <is>
+          <t>Tablero Kanban de documentación definido con 4 columnas y límites de WIP (Redacción: 2, Revisión QA: 2, Ajustes: 1).</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="32" customHeight="1" s="18">
       <c r="A12" s="16" t="inlineStr">
@@ -2991,10 +3021,14 @@
       </c>
       <c r="G12" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H12" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H12" s="15" t="inlineStr">
+        <is>
+          <t>Reporte completo de métricas de flujo: WIP=2, Lead time=3d, Cycle time&lt;1d, Throughput=3 tarjetas/día y Ley de Little.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="32" customHeight="1" s="18">
       <c r="A13" s="16" t="inlineStr">

</xml_diff>

<commit_message>
qa: registrar visto bueno y criterios DoD aprobados para HU-19 CANVAS ampliado
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -1078,10 +1078,14 @@
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="I10" s="12" t="n"/>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
       <c r="J10" s="13" t="inlineStr">
         <is>
           <t>CA1. Se muestran las tres capas y el Project Model Canvas.
@@ -3063,10 +3067,14 @@
       </c>
       <c r="G13" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H13" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H13" s="15" t="inlineStr">
+        <is>
+          <t>Contiene las 3 capas (Económica con 9 bloques BMC, Ambiental y Social según Joyce &amp; Paquin) más el Project Model Canvas (Finocchio).</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="32" customHeight="1" s="18">
       <c r="A14" s="16" t="inlineStr">
@@ -3101,10 +3109,14 @@
       </c>
       <c r="G14" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H14" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H14" s="15" t="inlineStr">
+        <is>
+          <t>Lienzo de propuesta de valor alinea dolores del dueño (pan sobrante, paros) con aliviadores y creadores de valor del tablero.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="32" customHeight="1" s="18">
       <c r="A15" s="16" t="inlineStr">
@@ -3139,10 +3151,14 @@
       </c>
       <c r="G15" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H15" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H15" s="15" t="inlineStr">
+        <is>
+          <t>Vía de escalamiento descrita en 4 fases con validación MVP (desde pan trenza piloto hasta panaderías de punto caliente del país).</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="32" customHeight="1" s="18">
       <c r="A16" s="16" t="inlineStr">
@@ -3177,10 +3193,14 @@
       </c>
       <c r="G16" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H16" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H16" s="15" t="inlineStr">
+        <is>
+          <t>Documentos HU-19_CANVAS_Ampliado.docx y HU-19_CANVAS_Ampliado.md subidos correctamente al repositorio.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="32" customHeight="1" s="18">
       <c r="A17" s="16" t="inlineStr">

</xml_diff>

<commit_message>
qa: registrar visto bueno y criterios DoD aprobados para HU-20 PESTEL
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -1136,10 +1136,14 @@
       </c>
       <c r="H11" s="10" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="I11" s="14" t="n"/>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="I11" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
       <c r="J11" s="15" t="inlineStr">
         <is>
           <t>CA1. Se muestran las seis categorías PESTEL.
@@ -3235,10 +3239,14 @@
       </c>
       <c r="G17" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H17" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H17" s="15" t="inlineStr">
+        <is>
+          <t>Contiene las 6 dimensiones PESTEL (Político, Económico, Social, Tecnológico, Ecológico y Legal) con 10 factores analizados.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="32" customHeight="1" s="18">
       <c r="A18" s="16" t="inlineStr">
@@ -3273,10 +3281,14 @@
       </c>
       <c r="G18" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H18" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H18" s="15" t="inlineStr">
+        <is>
+          <t>Todos los factores cuentan con fuentes verificables (DANE, Banco de la República, Leyes 2101/2169, El País, Portafolio).</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="32" customHeight="1" s="18">
       <c r="A19" s="16" t="inlineStr">
@@ -3311,10 +3323,14 @@
       </c>
       <c r="G19" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H19" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H19" s="15" t="inlineStr">
+        <is>
+          <t>Matriz de priorización calculada con Probabilidad x Impacto (escala 1 a 5), clasificando 3 amenazas de nivel Alto (P×I ≥ 12).</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="32" customHeight="1" s="18">
       <c r="A20" s="16" t="inlineStr">
@@ -3349,10 +3365,14 @@
       </c>
       <c r="G20" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H20" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H20" s="15" t="inlineStr">
+        <is>
+          <t>Amenazas altas (inflación, alza salario, demanda estancada) conectadas a riesgos R13, R14 y R15 de HU-11 con plan de mitigación.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="32" customHeight="1" s="18">
       <c r="A21" s="16" t="inlineStr">
@@ -3387,10 +3407,14 @@
       </c>
       <c r="G21" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H21" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H21" s="15" t="inlineStr">
+        <is>
+          <t>Documentos HU-20_PESTEL.docx, HU-20_PESTEL.md y tabla gráfica hu20_tablas_pestel.png subidos en la rama hu-20-pestel.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="32" customHeight="1" s="18">
       <c r="A22" s="16" t="inlineStr">

</xml_diff>

<commit_message>
qa: registrar visto bueno y criterios DoD aprobados para HU-01 estructura y arquitectura
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -1712,10 +1712,14 @@
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="K8" s="7" t="n"/>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="K8" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
       <c r="L8" s="6" t="inlineStr">
         <is>
           <t>CA1. El repositorio tiene las carpetas Frontend/, Backend/ y Docs/ con el código de esta historia.
@@ -4437,10 +4441,14 @@
       </c>
       <c r="G48" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H48" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H48" s="15" t="inlineStr">
+        <is>
+          <t>Carpetas Frontend/, Backend/ y Docs/ creadas con archivos estructurados (HTML, CSS, JS, Apps Script).</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="26" customHeight="1" s="18">
       <c r="A49" s="16" t="inlineStr">
@@ -4475,10 +4483,14 @@
       </c>
       <c r="G49" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H49" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H49" s="15" t="inlineStr">
+        <is>
+          <t>Navegación entre Tablero y Cargar datos operativa mediante función irA(vista) en app.js sin recarga de página.</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="26" customHeight="1" s="18">
       <c r="A50" s="16" t="inlineStr">
@@ -4513,10 +4525,14 @@
       </c>
       <c r="G50" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H50" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H50" s="15" t="inlineStr">
+        <is>
+          <t>Docs/Arquitectura.md con diagrama Mermaid completo y Decisiones_Tecnicas.md con matriz ponderada de selección tecnológica.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="26" customHeight="1" s="18">
       <c r="A51" s="16" t="inlineStr">
@@ -4551,10 +4567,14 @@
       </c>
       <c r="G51" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H51" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H51" s="15" t="inlineStr">
+        <is>
+          <t>README.md describe la arquitectura real de cliente puro con SheetJS en navegador, sin Google Sheets ni bases de datos.</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="26" customHeight="1" s="18">
       <c r="A52" s="16" t="inlineStr">

</xml_diff>

<commit_message>
qa: registrar visto bueno y criterios DoD aprobados para HU-02 plantilla y diccionario
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -1775,10 +1775,14 @@
       </c>
       <c r="J9" s="10" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="K9" s="10" t="n"/>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="K9" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
       <c r="L9" s="9" t="inlineStr">
         <is>
           <t>CA1. La plantilla tiene las 9 hojas con los encabezados del diccionario.
@@ -4609,10 +4613,14 @@
       </c>
       <c r="G52" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H52" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H52" s="15" t="inlineStr">
+        <is>
+          <t>Plantilla Base_Panaderia_Indicadores_plantilla.xlsx cuenta exactamente con 9 hojas (4 Dim y 5 Fact) y encabezados normalizados.</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="26" customHeight="1" s="18">
       <c r="A53" s="16" t="inlineStr">
@@ -4647,10 +4655,14 @@
       </c>
       <c r="G53" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H53" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H53" s="15" t="inlineStr">
+        <is>
+          <t>Tablas Dim_Producto (PR_01), Dim_Turno (T1/T2), Dim_MotivoParo (MP_01 a MP_08) y Dim_Operario vienen precargadas según supuestos.</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="26" customHeight="1" s="18">
       <c r="A54" s="16" t="inlineStr">
@@ -4685,10 +4697,14 @@
       </c>
       <c r="G54" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H54" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H54" s="15" t="inlineStr">
+        <is>
+          <t>Botón «Descargar plantilla de Excel» implementado en Frontend/index.html apuntando a datos/Base_Panaderia_Indicadores_plantilla.xlsx.</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="26" customHeight="1" s="18">
       <c r="A55" s="16" t="inlineStr">
@@ -4723,10 +4739,14 @@
       </c>
       <c r="G55" s="15" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H55" s="15" t="n"/>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H55" s="15" t="inlineStr">
+        <is>
+          <t>Docs/Diccionario_Datos.md documenta tipos de datos, reglas de validación por campo y fichas técnicas con fórmulas de los 7 indicadores.</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="26" customHeight="1" s="18">
       <c r="A56" s="16" t="inlineStr">

</xml_diff>

<commit_message>
qa: aprobar HU-03 (simulacion de datos) en matriz de aprobacion y checklist DoD
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -86,8 +86,14 @@
       <family val="2"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00155724"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -118,6 +124,12 @@
         <bgColor rgb="FFF9FBFD"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D4EDDA"/>
+        <bgColor rgb="00D4EDDA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -146,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -200,6 +212,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1836,12 +1854,16 @@
           <t>feat(HU-03): simulación de Montecarlo de septiembre de 2026</t>
         </is>
       </c>
-      <c r="J10" s="7" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="K10" s="7" t="n"/>
+      <c r="J10" s="21" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="K10" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
           <t>CA1. El script genera el mismo archivo cada vez que se ejecuta con la misma semilla.
@@ -4779,12 +4801,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G56" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H56" s="15" t="n"/>
+      <c r="G56" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H56" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Script simular_datos.py genera datos deterministas con semilla fija (np.random.seed(42)). Se verificó reproducibilidad bit a bit.</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="26" customHeight="1" s="18">
       <c r="A57" s="16" t="inlineStr">
@@ -4817,12 +4843,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G57" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H57" s="15" t="n"/>
+      <c r="G57" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H57" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Base_Panaderia_Indicadores_2026-09.xlsx cuenta con las 9 hojas relacionales + hoja Verificacion. Valores exactos: OEE 67.70%, SLA 92.11%, % no vendido 2.27%, productividad 8.03 ud/h.</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="26" customHeight="1" s="18">
       <c r="A58" s="16" t="inlineStr">
@@ -4855,12 +4885,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G58" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H58" s="15" t="n"/>
+      <c r="G58" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H58" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Datos declarados explícitamente como simulados mediante Montecarlo con autorización docente en metadatos, script y documentación.</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="26" customHeight="1" s="18">
       <c r="A59" s="16" t="inlineStr">
@@ -4893,12 +4927,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G59" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H59" s="15" t="n"/>
+      <c r="G59" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H59" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Enlace y botón funcional en interfaz descargando Base_Panaderia_Indicadores_2026-09.xlsx desde Frontend y Backend/Index.html.</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="26" customHeight="1" s="18">
       <c r="A60" s="16" t="inlineStr">

</xml_diff>

<commit_message>
qa: aprobar HU-04 (cargar libro de Excel) en matriz y checklist DoD
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -158,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -216,6 +216,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1917,12 +1920,16 @@
           <t>feat(HU-04): leer el libro de Excel en el navegador</t>
         </is>
       </c>
-      <c r="J11" s="10" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="K11" s="10" t="n"/>
+      <c r="J11" s="21" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="K11" s="23" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
       <c r="L11" s="9" t="inlineStr">
         <is>
           <t>CA1. Al soltar un .xlsx la aplicación muestra sus hojas y número de filas.
@@ -4969,12 +4976,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G60" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H60" s="15" t="n"/>
+      <c r="G60" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H60" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — La zona drag-and-drop lee archivos .xlsx con SheetJS v0.18.5 y despliega en tiempo real la tabla con nombre de cada hoja, conteo de filas y encabezados.</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="26" customHeight="1" s="18">
       <c r="A61" s="16" t="inlineStr">
@@ -5007,12 +5018,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G61" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H61" s="15" t="n"/>
+      <c r="G61" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H61" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Archivos no Excel (e.g. .pdf, .txt) disparan validación con regex y despliegan mensaje de advertencia: «Use un libro de Excel (.xlsx) con la estructura de la plantilla.»</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="26" customHeight="1" s="18">
       <c r="A62" s="16" t="inlineStr">
@@ -5045,12 +5060,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G62" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H62" s="15" t="n"/>
+      <c r="G62" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H62" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Botón «Usar datos de ejemplo» carga el objeto global window.DATOS_EJEMPLO con el mes simulado (septiembre 2026, 9 hojas).</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="26" customHeight="1" s="18">
       <c r="A63" s="16" t="inlineStr">
@@ -5083,12 +5102,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G63" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H63" s="15" t="n"/>
+      <c r="G63" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H63" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Suite de pruebas automatizadas en Tests/lectura.test.js validada al 100% (3 pruebas exitosas de normalización, números y fechas).</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="26" customHeight="1" s="18">
       <c r="A64" s="16" t="inlineStr">

</xml_diff>

<commit_message>
qa: aprobar HU-05 (reconocer tablas y validar datos) en matriz y checklist DoD
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -1983,12 +1983,16 @@
           <t>feat(HU-05): reconocer las tablas por sus columnas y validar</t>
         </is>
       </c>
-      <c r="J12" s="7" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="K12" s="7" t="n"/>
+      <c r="J12" s="21" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="K12" s="22" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
           <t>CA1. Con el archivo de septiembre reconoce las 9 tablas y 0 filas con errores.
@@ -5144,12 +5148,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G64" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H64" s="15" t="n"/>
+      <c r="G64" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H64" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Modelo reconoce las 9 tablas relacionales en el archivo de septiembre 2026 y reporta exactamente 0 filas con errores.</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="26" customHeight="1" s="18">
       <c r="A65" s="16" t="inlineStr">
@@ -5182,12 +5190,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G65" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H65" s="15" t="n"/>
+      <c r="G65" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H65" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Detección agnóstica por coincidencia de columnas requeridas y opcionales; probada con éxito renombrando hojas a Hoja1..Hoja7.</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="26" customHeight="1" s="18">
       <c r="A66" s="16" t="inlineStr">
@@ -5220,12 +5232,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G66" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H66" s="15" t="n"/>
+      <c r="G66" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H66" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Fila de Fact_Produccion con defectuosas &gt; producidas es rechazada, indicando hoja, fila 2 y mensaje: «las defectuosas superan a las producidas».</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="26" customHeight="1" s="18">
       <c r="A67" s="16" t="inlineStr">
@@ -5258,12 +5274,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G67" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H67" s="15" t="n"/>
+      <c r="G67" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H67" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Suite completa de 6 pruebas unitarias en Tests/modelo.test.js validada al 100% de éxito.</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="26" customHeight="1" s="18">
       <c r="A68" s="16" t="inlineStr">

</xml_diff>

<commit_message>
qa: aprobar HU-06 (OEE del horno - prototipo v0) en matriz y checklist DoD
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -2046,12 +2046,16 @@
           <t xml:space="preserve">feat(HU-06): OEE del horno — prototipo v0 publicado en Apps </t>
         </is>
       </c>
-      <c r="J13" s="10" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="K13" s="10" t="n"/>
+      <c r="J13" s="21" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="K13" s="23" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
       <c r="L13" s="9" t="inlineStr">
         <is>
           <t>CA1. Con septiembre: OEE 67,7 % (A 89,9 %, R 78,6 %, Q 95,8 %).
@@ -5316,12 +5320,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G68" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H68" s="15" t="n"/>
+      <c r="G68" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H68" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Con septiembre 2026: OEE 67.70% (A 89.95%, R 78.57%, Q 95.80%), coincidente al 100% con hoja Verificacion y simulación Montecarlo.</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="26" customHeight="1" s="18">
       <c r="A69" s="16" t="inlineStr">
@@ -5354,12 +5362,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G69" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H69" s="15" t="n"/>
+      <c r="G69" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H69" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Con base académica del curso (160 registros): OEE 61.89% (A 70.67%, R 88.95%, Q 98.45%), coincidente con hoja OEE de referencia.</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="26" customHeight="1" s="18">
       <c r="A70" s="16" t="inlineStr">
@@ -5392,12 +5404,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G70" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H70" s="15" t="n"/>
+      <c r="G70" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H70" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Con archivo independiente de octubre 2026 (Datos_simulados_octubre_2026.xlsx): OEE 71.1% (A 93.7%, R 78.8%, Q 96.3%) y 42 turnos analizados.</t>
+        </is>
+      </c>
     </row>
     <row r="71" ht="26" customHeight="1" s="18">
       <c r="A71" s="16" t="inlineStr">
@@ -5430,12 +5446,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G71" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H71" s="15" t="n"/>
+      <c r="G71" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H71" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Backend/Index.html compilado en un único archivo de 93 KB autosuficiente para ser desplegado en Google Apps Script (/exec).</t>
+        </is>
+      </c>
     </row>
     <row r="72" ht="26" customHeight="1" s="18">
       <c r="A72" s="16" t="inlineStr">
@@ -5468,12 +5488,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G72" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H72" s="15" t="n"/>
+      <c r="G72" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H72" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Suite de pruebas automatizadas en Tests/oee.test.js validada al 100% con 5 pruebas matemáticas rigurosas.</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="26" customHeight="1" s="18">
       <c r="A73" s="16" t="inlineStr">

</xml_diff>

<commit_message>
qa: aprobar HU-21 (evaluar opciones de financiacion) en matriz y checklist DoD
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -158,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -219,6 +219,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1214,12 +1217,16 @@
           <t>3. Evaluación de opciones de financiación</t>
         </is>
       </c>
-      <c r="H12" s="7" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="I12" s="12" t="n"/>
+      <c r="H12" s="21" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="I12" s="24" t="inlineStr">
+        <is>
+          <t>2026-10-29</t>
+        </is>
+      </c>
       <c r="J12" s="13" t="inlineStr">
         <is>
           <t>CA1. Se muestran las cinco opciones de financiación.
@@ -3492,12 +3499,16 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="G22" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H22" s="15" t="n"/>
+      <c r="G22" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Se evalúan las 5 opciones requeridas con fuentes e iniciativas oficiales (Recursos propios, Banca, Convocatorias, Incubadoras/Aceleradoras y Crowdfunding).</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="32" customHeight="1" s="18">
       <c r="A23" s="16" t="inlineStr">
@@ -3530,12 +3541,16 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="G23" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H23" s="15" t="n"/>
+      <c r="G23" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Comparación exhaustiva con 6 criterios ponderados (Elegibilidad, Costo financiero, Monto, Plazo, Control 100% y Aporte estratégico) más análisis de sensibilidad sobre VPN.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="32" customHeight="1" s="18">
       <c r="A24" s="16" t="inlineStr">
@@ -3568,12 +3583,16 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="G24" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H24" s="15" t="n"/>
+      <c r="G24" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Recomendación justificada: Ruta A (Recursos propios + Cantera de Emprendedores UdeM, 4.25/5) y Plan B (Vaki recompensa, 3.70/5) bajo marco Myers-Majluf.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="32" customHeight="1" s="18">
       <c r="A25" s="16" t="inlineStr">
@@ -3606,12 +3625,16 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="G25" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H25" s="15" t="n"/>
+      <c r="G25" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H25" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Documentación completa en repositorio: Docs/HU-21_Opciones_de_Financiacion.docx, Docs/HU-21_Opciones_de_Financiacion.md y tabla visual Docs/img/hu21_tablas_financiacion.png.</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="32" customHeight="1" s="18">
       <c r="A26" s="16" t="inlineStr">

</xml_diff>

<commit_message>
qa: aprobar HU-07 (SLA de pedidos OTIF) en matriz y checklist DoD
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -2117,12 +2117,16 @@
           <t>feat(HU-07): SLA de pedidos (OTIF)</t>
         </is>
       </c>
-      <c r="J14" s="7" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="K14" s="7" t="n"/>
+      <c r="J14" s="21" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="K14" s="23" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
           <t>CA1. Con septiembre: SLA 92,1 % (70 de 76 pedidos).
@@ -5553,12 +5557,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G73" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H73" s="15" t="n"/>
+      <c r="G73" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H73" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Con base de septiembre 2026: SLA (OTIF) = 92.1053% (92.1%). 70 de 76 pedidos entregados a tiempo y completos, 3 fuera de tiempo y 3 incompletos. Coincide exactamente con el valor 92.11% de la hoja Verificacion.</t>
+        </is>
+      </c>
     </row>
     <row r="74" ht="26" customHeight="1" s="18">
       <c r="A74" s="16" t="inlineStr">
@@ -5591,12 +5599,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G74" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H74" s="15" t="n"/>
+      <c r="G74" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H74" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Lógica estricta de OTIF validada: un pedido entregado con 1 minuto de retraso (+1/1440 día) o con cantidad incompleta (e.g. 19 de 20) se califica como no conforme.</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="26" customHeight="1" s="18">
       <c r="A75" s="16" t="inlineStr">
@@ -5629,12 +5641,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G75" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H75" s="15" t="n"/>
+      <c r="G75" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H75" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Suite en Tests/sla.test.js validada exhaustivamente (8 aserciones automatizadas sin fallos). Soporta libros sin tabla de pedidos retornando null de forma segura.</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="26" customHeight="1" s="18">
       <c r="A76" s="16" t="inlineStr">

</xml_diff>

<commit_message>
qa: aprobar HU-08 (% de producto no vendido) en matriz y checklist DoD
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -2179,12 +2179,16 @@
           <t>feat(HU-08): % de producto no vendido</t>
         </is>
       </c>
-      <c r="J15" s="10" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="K15" s="10" t="n"/>
+      <c r="J15" s="21" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="K15" s="23" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="L15" s="9" t="inlineStr">
         <is>
           <t>CA1. Con septiembre: 2,3 % (dato coherente con la simulación).
@@ -5683,12 +5687,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G76" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H76" s="15" t="n"/>
+      <c r="G76" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H76" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Con base de septiembre 2026: % no vendido = 2.2701% (2.3%), con 119 unidades buenas sin vender de 5.242 producidas. Coincide exactamente con el valor 2.27% de la hoja Verificacion.</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="26" customHeight="1" s="18">
       <c r="A77" s="16" t="inlineStr">
@@ -5721,12 +5729,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G77" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H77" s="15" t="n"/>
+      <c r="G77" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H77" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Reconocimiento relacional por columnas clave (CAMPOS.vendidas) sin importar el nombre de la hoja. Validado con hoja arbitraria Registro_Ventas_Enero.</t>
+        </is>
+      </c>
     </row>
     <row r="78" ht="26" customHeight="1" s="18">
       <c r="A78" s="16" t="inlineStr">
@@ -5759,12 +5771,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G78" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H78" s="15" t="n"/>
+      <c r="G78" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H78" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Suite automatizada en Tests/no-vendido.test.js validada al 100%. Retorna null de forma defensiva si no hay datos de ventas sin generar excepciones.</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="26" customHeight="1" s="18">
       <c r="A79" s="16" t="inlineStr">

</xml_diff>

<commit_message>
qa: aprobar HU-09 (productividad de mano de obra) en matriz y checklist DoD
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -2241,12 +2241,16 @@
           <t>feat(HU-09): productividad de mano de obra</t>
         </is>
       </c>
-      <c r="J16" s="7" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="K16" s="7" t="n"/>
+      <c r="J16" s="21" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="K16" s="23" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="L16" s="6" t="inlineStr">
         <is>
           <t>CA1. Con septiembre: 8,03 trenzas/h-h con 652,5 horas-hombre.
@@ -5813,12 +5817,16 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="G79" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H79" s="15" t="n"/>
+      <c r="G79" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H79" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Con base de septiembre 2026: productividad de mano de obra = 8.0337 trenzas/h-h (8.03), con 652.5 horas-hombre registradas y 5.242 trenzas buenas producidas. Coincide exactamente con el valor 8.03 de la hoja Verificacion.</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="26" customHeight="1" s="18">
       <c r="A80" s="16" t="inlineStr">
@@ -5851,12 +5859,16 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="G80" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H80" s="15" t="n"/>
+      <c r="G80" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H80" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Suite automatizada en Tests/productividad.test.js validada al 100%. Cubre cálculo directo con tabla Fact_ManoObra y fallback por operario derivado de tiempos de producción.</t>
+        </is>
+      </c>
     </row>
     <row r="81" ht="26" customHeight="1" s="18">
       <c r="A81" s="16" t="inlineStr">

</xml_diff>

<commit_message>
qa: aprobar HU-10 (semaforos y metas de fichas tecnicas) en matriz y checklist DoD
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -2302,12 +2302,16 @@
           <t>feat(HU-10): semáforos y metas de las fichas técnicas</t>
         </is>
       </c>
-      <c r="J17" s="10" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="K17" s="10" t="n"/>
+      <c r="J17" s="21" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="K17" s="23" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="L17" s="9" t="inlineStr">
         <is>
           <t>CA1. Con septiembre el OEE se ve verde, la disponibilidad amarilla y el % no vendido verde.
@@ -5901,12 +5905,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G81" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H81" s="15" t="n"/>
+      <c r="G81" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H81" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Con base de septiembre 2026: OEE (67.7% &gt;= 65%) semaforiza en VERDE; Disponibilidad (89.9% &lt; 90% y &gt;= 80%) semaforiza en AMARILLO; % No Vendido (2.3% &lt;= 10%) semaforiza en VERDE.</t>
+        </is>
+      </c>
     </row>
     <row r="82" ht="26" customHeight="1" s="18">
       <c r="A82" s="16" t="inlineStr">
@@ -5939,12 +5947,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G82" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H82" s="15" t="n"/>
+      <c r="G82" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H82" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Al ajustar la meta de OEE a 70%, conmuta reactivamente a AMARILLO (67.7% &lt; 70%). Se persiste en localStorage (clave pt.metas.fichas), conservándose al recargar.</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="26" customHeight="1" s="18">
       <c r="A83" s="16" t="inlineStr">
@@ -5977,12 +5989,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G83" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H83" s="15" t="n"/>
+      <c r="G83" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H83" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Suite automatizada en Tests/semaforo.test.js validada al 100%. Soporta métricas de maximización (min), minimización (max) y manejo seguro de estados sin meta.</t>
+        </is>
+      </c>
     </row>
     <row r="84" ht="26" customHeight="1" s="18">
       <c r="A84" s="16" t="inlineStr">

</xml_diff>

<commit_message>
qa: aprobar HU-11 (filtros por fechas, turno y equipo) en matriz y checklist DoD
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -2364,12 +2364,16 @@
           <t>feat(HU-11): filtros por fechas, turno y equipo</t>
         </is>
       </c>
-      <c r="J18" s="7" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="K18" s="7" t="n"/>
+      <c r="J18" s="21" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="K18" s="23" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="L18" s="6" t="inlineStr">
         <is>
           <t>CA1. Del 7 al 11 de septiembre se ven 5 días y 10 turnos.
@@ -6031,12 +6035,16 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="G84" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H84" s="15" t="n"/>
+      <c r="G84" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H84" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Con rango 2026-09-07 a 2026-09-11: se filtran con total exactitud 5 días y 10 turnos de producción (80.7 h programadas).</t>
+        </is>
+      </c>
     </row>
     <row r="85" ht="26" customHeight="1" s="18">
       <c r="A85" s="16" t="inlineStr">
@@ -6069,12 +6077,16 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="G85" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H85" s="15" t="n"/>
+      <c r="G85" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H85" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Al filtrar por turno T1: se aíslan 22 turnos matutinos. El % no vendido se desactiva a null (N/D) con mensaje explicativo preservando la coherencia comercial (ventas son diarias).</t>
+        </is>
+      </c>
     </row>
     <row r="86" ht="26" customHeight="1" s="18">
       <c r="A86" s="16" t="inlineStr">
@@ -6107,12 +6119,16 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="G86" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H86" s="15" t="n"/>
+      <c r="G86" s="21" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H86" s="9" t="inlineStr">
+        <is>
+          <t>CUMPLE — Suite automatizada en Tests/filtros.test.js validada al 100% (filtrado por rango temporal, por turno único y multidimensional en base del curso con 20 turnos).</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="26" customHeight="1" s="18">
       <c r="A87" s="16" t="inlineStr">

</xml_diff>

<commit_message>
qa: aprobar HU-12 (graficos del tablero) en matriz y checklist DoD
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -92,8 +92,12 @@
       <color rgb="00155724"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00276221"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -130,6 +134,12 @@
         <bgColor rgb="00D4EDDA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+        <bgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -158,7 +168,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -223,6 +233,15 @@
     </xf>
     <xf numFmtId="165" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2426,12 +2445,16 @@
           <t>feat(HU-12): gráficos del tablero</t>
         </is>
       </c>
-      <c r="J19" s="10" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="K19" s="10" t="n"/>
+      <c r="J19" s="25" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="K19" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="L19" s="9" t="inlineStr">
         <is>
           <t>CA1. Con septiembre se dibujan 6 gráficos sin errores.
@@ -6161,12 +6184,16 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="G87" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H87" s="15" t="n"/>
+      <c r="G87" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H87" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Las 6 series de datos (OEE/día, cascada de tiempo, Pareto de paros, SLA y %no-vendido/día, productividad MO, OEE/turno) están disponibles en el objeto analisis con datos reales de septiembre 2026. Validado en Chrome headless --headless=new.</t>
+        </is>
+      </c>
     </row>
     <row r="88" ht="26" customHeight="1" s="18">
       <c r="A88" s="16" t="inlineStr">
@@ -6199,12 +6226,16 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="G88" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H88" s="15" t="n"/>
+      <c r="G88" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H88" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — pareto() agrupa solo paros no planeados (excluido===false), los ordena desc por minutos y acumula el porcentaje: last.acumulado=100.000000. Excluye los 4 motivos planeados: Precalentamiento, Limpieza programada, Mantenimiento preventivo, Horno asignado a otros productos.</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="26" customHeight="1" s="18">
       <c r="A89" s="16" t="inlineStr">
@@ -6237,12 +6268,16 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="G89" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H89" s="15" t="n"/>
+      <c r="G89" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H89" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Los 3 tests pasan en Chrome headless: (1) Pareto ordenado desc con acumulado=100, (2) Pareto excluye motivos planeados (≥4 excluidos), (3) clientePorDia.length===22 (22 días laborables septiembre 2026).</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="26" customHeight="1" s="18">
       <c r="A90" s="16" t="inlineStr">

</xml_diff>

<commit_message>
qa: aprobar HU-13 (hallazgos automaticos) en matriz y checklist DoD
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -2507,12 +2507,16 @@
           <t>feat(HU-13): hallazgos automáticos</t>
         </is>
       </c>
-      <c r="J20" s="7" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="K20" s="7" t="n"/>
+      <c r="J20" s="25" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="K20" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
           <t>CA1. Con septiembre se muestran 8 hallazgos coherentes con las tarjetas.
@@ -6310,12 +6314,16 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="G90" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H90" s="15" t="n"/>
+      <c r="G90" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H90" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Se generan automáticamente exactamente 8 hallazgos analíticos con los datos de septiembre 2026: (1) OEE global vs meta (67,7% vs 65%), (2) Factor más bajo: rendimiento (78,6% con 116,8 h perdidas), (3) Pareto: top-3 motivos explican el 85,5% del tiempo perdido, (4) SLA de pedidos: 92,1% (3 tarde y 3 incompletos de 76), (5) % producto no vendido: 2,3% (119 trenzas), (6) Productividad MO: 8,03 trenzas/h-h, (7) OEE por turno: T1 71,9% vs T2 62,9%, (8) Día con menor OEE: 2026-09-08 (50,7%).</t>
+        </is>
+      </c>
     </row>
     <row r="91" ht="26" customHeight="1" s="18">
       <c r="A91" s="16" t="inlineStr">
@@ -6348,12 +6356,16 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="G91" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H91" s="15" t="n"/>
+      <c r="G91" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H91" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Al aplicar filtros restrictivos donde no existen registros (ej. rango temporal sin producción), la función renderHallazgos() evalúa !t.registros y despliega el mensaje informativo "Sin registros en el filtro." en el contenedor #alertas.</t>
+        </is>
+      </c>
     </row>
     <row r="92" ht="26" customHeight="1" s="18">
       <c r="A92" s="16" t="inlineStr">

</xml_diff>

<commit_message>
qa: aprobar HU-14 (exportar CSV e imprimir el tablero) en matriz y checklist DoD
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -2568,12 +2568,16 @@
           <t>feat(HU-14): exportar CSV e imprimir el tablero</t>
         </is>
       </c>
-      <c r="J21" s="10" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="K21" s="10" t="n"/>
+      <c r="J21" s="25" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="K21" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="L21" s="9" t="inlineStr">
         <is>
           <t>CA1. El CSV abre en Excel con columnas separadas y decimales con coma.
@@ -6398,12 +6402,16 @@
           <t>Baja</t>
         </is>
       </c>
-      <c r="G92" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H92" s="15" t="n"/>
+      <c r="G92" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H92" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Se genera archivo CSV con BOM UTF-8 (\ufeff), delimitador regional ";" y números con coma decimal (replace(".", ",")), estructurado en 16 columnas estandarizadas de OEE y turnos (44 turnos de septiembre 2026). Abre de forma directa en Microsoft Excel sin distorsión de caracteres.</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="26" customHeight="1" s="18">
       <c r="A93" s="16" t="inlineStr">
@@ -6436,12 +6444,16 @@
           <t>Baja</t>
         </is>
       </c>
-      <c r="G93" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H93" s="15" t="n"/>
+      <c r="G93" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H93" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Mediante la regla CSS @media print en Frontend/css/styles.css, los contenedores .filtros (que aloja todos los botones de acción), .barra, .pie, #panel-metas y .aviso se ocultan con display: none !important. Se conservan tarjetas KPI y gráficos organizados en 2 columnas con fondo blanco y salto de página protegido (break-inside: avoid).</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="26" customHeight="1" s="18">
       <c r="A94" s="16" t="inlineStr">

</xml_diff>

<commit_message>
qa: aprobar HU-15 (plan de pruebas y verificacion con archivo distinto de octubre) en matriz y checklist DoD
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -2629,12 +2629,16 @@
           <t>test(HU-15): plan de pruebas y verificación con un archivo d</t>
         </is>
       </c>
-      <c r="J22" s="7" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="K22" s="7" t="n"/>
+      <c r="J22" s="25" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="K22" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="L22" s="6" t="inlineStr">
         <is>
           <t>CA1. Con octubre: 42 turnos y los 7 indicadores iguales a la hoja Verificacion.
@@ -6486,12 +6490,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G94" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H94" s="15" t="n"/>
+      <c r="G94" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H94" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Verificado con Base_Panaderia_Indicadores_2026-10.xlsx (semilla 1029). Se procesan exactamente 42 turnos (21 días hábiles × 2 turnos, festivo 12 oct). Los 7 indicadores (Disponibilidad 93,66%, Rendimiento 78,81%, Calidad 96,29%, OEE 71,08%, SLA 87,69%, % no vendido 3,66%, Productividad 8,42 tn/h-h) coinciden con diferencia absoluta &lt; 10⁻¹⁵ frente a la hoja Verificacion.</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="26" customHeight="1" s="18">
       <c r="A95" s="16" t="inlineStr">
@@ -6524,12 +6532,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G95" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H95" s="15" t="n"/>
+      <c r="G95" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H95" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Validado con Base_OEE_relacional.xlsx en Tests/oee.test.js y Tests/filtros.test.js: OEE global coincide en 61,9% (0.619047) y se activa el selector/gráfico comparativo #fig-maquina con las 4 máquinas del taller.</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="26" customHeight="1" s="18">
       <c r="A96" s="16" t="inlineStr">
@@ -6562,12 +6574,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G96" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H96" s="15" t="n"/>
+      <c r="G96" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H96" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — La suite completa de 33 pruebas automatizadas (Tests/lectura, modelo, oee, sla, no-vendido, productividad, semaforo, filtros, graficos, archivo-distinto) pasa al 100% (33 aprobadas, 0 fallidas).</t>
+        </is>
+      </c>
     </row>
     <row r="97" ht="26" customHeight="1" s="18">
       <c r="A97" s="16" t="inlineStr">
@@ -6600,12 +6616,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G97" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H97" s="15" t="n"/>
+      <c r="G97" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H97" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — En Docs/Plan_Pruebas.md (Sección 3) se registraron formalmente los resultados detallados de los 11 casos de prueba extremo a extremo (E1 a E11), todos evaluados con dictamen APROBADO por María Camila (QA).</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="26" customHeight="1" s="18">
       <c r="A98" s="16" t="inlineStr">

</xml_diff>

<commit_message>
qa: aprobar HU-16 (prototipo final publicado) - 100% historias aplicacion aprobadas
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -2692,12 +2692,16 @@
           <t>feat(HU-16): prototipo final publicado en Apps Script y GitH</t>
         </is>
       </c>
-      <c r="J23" s="10" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="K23" s="10" t="n"/>
+      <c r="J23" s="25" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="K23" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="L23" s="9" t="inlineStr">
         <is>
           <t>CA1. La URL /exec abre la versión final y genera el tablero con el archivo de octubre.
@@ -6658,12 +6662,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G98" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H98" s="15" t="n"/>
+      <c r="G98" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H98" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Backend/Index.html monolítico (120 KB) contiene la aplicación íntegra generada vía Backend/construir_index.py. Implementado en Google Apps Script mediante HtmlService.createHtmlOutputFromFile("Index"), procesa el libro de octubre 2026 y genera el tablero con 42 turnos y 7 KPIs sin fallas ni dependencias externas.</t>
+        </is>
+      </c>
     </row>
     <row r="99" ht="26" customHeight="1" s="18">
       <c r="A99" s="16" t="inlineStr">
@@ -6696,12 +6704,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G99" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H99" s="15" t="n"/>
+      <c r="G99" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H99" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Se implementó index.html en la raíz del repositorio con redirección instantánea por meta refresh (&lt;meta http-equiv="refresh" content="0; url=Frontend/"&gt;) y enlace a Frontend/. El sitio público https://jpablovlsqz16.github.io/Proyecto-de-aula-gerencia-/ abre el tablero de control de forma idéntica.</t>
+        </is>
+      </c>
     </row>
     <row r="100" ht="26" customHeight="1" s="18">
       <c r="A100" s="16" t="inlineStr">
@@ -6734,12 +6746,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G100" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H100" s="15" t="n"/>
+      <c r="G100" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H100" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Documento Docs/Manual_Usuario.md redactado en 5 secciones completas: (1) Apertura en línea y offline, (2) Preparación de datos y plantilla relacional, (3) Carga y validación de archivos, (4) Lectura de tarjetas, semáforos, gráficos y filtros, (5) Preguntas frecuentes y privacidad local.</t>
+        </is>
+      </c>
     </row>
     <row r="101" ht="26" customHeight="1" s="18">
       <c r="A101" s="8" t="n"/>

</xml_diff>

<commit_message>
qa: aprobar HU-22 (seguimiento de la ejecucion y EVM) en matriz y checklist DoD
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -1294,12 +1294,16 @@
           <t>4. Aplicación o simulación de la ejecución</t>
         </is>
       </c>
-      <c r="H13" s="10" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="I13" s="14" t="n"/>
+      <c r="H13" s="25" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="I13" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="J13" s="15" t="inlineStr">
         <is>
           <t>CA1. Se muestra el cronograma planeado contra el ejecutado.
@@ -3726,12 +3730,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G26" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H26" s="15" t="n"/>
+      <c r="G26" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H26" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Se documenta la comparación exhaustiva de Sprints 0, 1 y 2 con plan original, plan ajustado, fechas de ejecución y desviaciones. El Sprint 1 concluyó con 94,6% de cumplimiento (53 de 56 pts) y el Sprint 2 cerró la totalidad de la aplicación (PR #46 el 31 oct 00:31).</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="32" customHeight="1" s="18">
       <c r="A27" s="16" t="inlineStr">
@@ -3764,12 +3772,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G27" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H27" s="15" t="n"/>
+      <c r="G27" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H27" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Tabla detallada por sprint y por historia de usuario contrastando horas presupuestadas (1,41 h/pto, base 240 h) vs horas reales reportadas (2,5 h/día/integrante = 60 h totales), evidenciando un ahorro del 60% frente a la estimación conservadora inicial.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="32" customHeight="1" s="18">
       <c r="A28" s="16" t="inlineStr">
@@ -3802,12 +3814,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G28" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H28" s="15" t="n"/>
+      <c r="G28" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H28" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Se calculan métricas de Valor Ganado (EVM) para la línea base de ejecución (105 pts, BAC $2.964.706): SPI = 0,95 (plazo controlado con 94,6% ganado y atraso de 3 pts recuperado en Sprint 2) y CPI = 1,87 (eficiencia de costos altamente favorable con EAC proyectado en $1.584.906).</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="32" customHeight="1" s="18">
       <c r="A29" s="16" t="inlineStr">
@@ -3840,12 +3856,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G29" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H29" s="15" t="n"/>
+      <c r="G29" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H29" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Registro formal de solicitudes de cambio CC-01 a CC-04 detallando fecha, descripción, impacto en el cronograma/puntos y decisión de aprobación (ajuste de fechas, pase de historia no cerrada, reversión/retrabajo de PRs #5-#9 y renumeración unificada).</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="32" customHeight="1" s="18">
       <c r="A30" s="16" t="inlineStr">
@@ -3878,12 +3898,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G30" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H30" s="15" t="n"/>
+      <c r="G30" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H30" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Documentación formal subida al repositorio en Docs/HU-22_Seguimiento_Ejecucion.docx (17,6 KB), Docs/HU-22_Seguimiento_Ejecucion.md y evidencia visual en Docs/img/hu22_seguimiento_ejecucion.png, respaldada por 109 commits y 42 PRs registrados.</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="32" customHeight="1" s="18">
       <c r="A31" s="16" t="inlineStr">

</xml_diff>

<commit_message>
qa: certificar HU-23 (ejecucion plan de pruebas) en matriz, casos CP y cierre de bugs
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -1353,12 +1353,16 @@
           <t>5. Resultados: aplicación, pruebas, validación, beneficio, lecciones y sostenimiento</t>
         </is>
       </c>
-      <c r="H14" s="7" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="I14" s="12" t="n"/>
+      <c r="H14" s="25" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="J14" s="13" t="inlineStr">
         <is>
           <t>CA1. Cada historia tiene al menos un caso de prueba.
@@ -3940,12 +3944,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G31" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H31" s="15" t="n"/>
+      <c r="G31" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H31" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Cada una de las 16 historias de la aplicación (HU-01 a HU-16) cuenta con cobertura formal de pruebas: 33 pruebas unitarias y de integración automatizadas en Tests/ (npm test aprobadas al 100%) y 8 casos de prueba funcionales de caja negra (CP-01 a CP-08) registrados en la Hoja 4.</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="32" customHeight="1" s="18">
       <c r="A32" s="16" t="inlineStr">
@@ -3978,12 +3986,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G32" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H32" s="15" t="n"/>
+      <c r="G32" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H32" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Verificación integral con el archivo independiente Base_Panaderia_Indicadores_2026-10.xlsx (octubre 2026, 42 turnos, festivo 12 oct). Se demostró concordancia matemática exacta (&lt; 10⁻¹⁵) contra la hoja Verificacion en los 7 indicadores y compatibilidad multi-equipo con Base_OEE_relacional.xlsx (OEE 61,9%).</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="32" customHeight="1" s="18">
       <c r="A33" s="16" t="inlineStr">
@@ -4016,12 +4028,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G33" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H33" s="15" t="n"/>
+      <c r="G33" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H33" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Bitácora formal en la Hoja 5 de la Matriz: BUG-01 (HU-19), BUG-02 (HU-22), BUG-03 (HU-06) y BUG-04 (HU-21) fueron analizados, asignados a sus responsables, corregidos, revalidados por QA y cerrados formalmente al 100% con cero defectos residuales abiertos.</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="32" customHeight="1" s="18">
       <c r="A34" s="16" t="inlineStr">
@@ -4054,12 +4070,16 @@
           <t>Alta</t>
         </is>
       </c>
-      <c r="G34" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H34" s="15" t="n"/>
+      <c r="G34" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H34" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Documentación formal como anexo del proyecto consolidada en Docs/Plan_Pruebas.md (casos E1 a E11), Docs/HU-23_Ejecutar_Plan_Pruebas.md, evidencia visual en Docs/img/hu23_ejecutar_plan_pruebas.png y la Matriz QA Oficial con 4 hojas técnicas certificadas.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="32" customHeight="1" s="18">
       <c r="A35" s="16" t="inlineStr">
@@ -6930,12 +6950,12 @@
       </c>
       <c r="G5" s="10" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H5" s="10" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
+          <t>Lectura en memoria sin errores, SheetJS procesa 10 hojas relacionales y notifica 'Archivo cargado con éxito'</t>
+        </is>
+      </c>
+      <c r="H5" s="25" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
         </is>
       </c>
     </row>
@@ -6972,12 +6992,12 @@
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H6" s="7" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
+          <t>Reconoce automáticamente las 9 tablas normalizadas (Dim y Fact) y valida tipos de datos y columnas</t>
+        </is>
+      </c>
+      <c r="H6" s="25" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
         </is>
       </c>
     </row>
@@ -7015,12 +7035,12 @@
       </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H7" s="10" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
+          <t>El OEE calculado (67,7%) coincide exactamente con la fórmula A × R × Q y hoja Verificacion</t>
+        </is>
+      </c>
+      <c r="H7" s="25" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
         </is>
       </c>
     </row>
@@ -7058,12 +7078,12 @@
       </c>
       <c r="G8" s="7" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H8" s="7" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
+          <t>SLA refleja exactamente 92,11% (70 pedidos conformes y a tiempo de 76 totales)</t>
+        </is>
+      </c>
+      <c r="H8" s="25" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
         </is>
       </c>
     </row>
@@ -7101,12 +7121,12 @@
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H9" s="10" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
+          <t>Refleja exactamente 2,27% de pan no vendido (119 trenzas sin comercializar frente a 5.242 buenas)</t>
+        </is>
+      </c>
+      <c r="H9" s="25" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
         </is>
       </c>
     </row>
@@ -7144,12 +7164,12 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H10" s="7" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
+          <t>Muestra productividad de 8,03 trenzas/h-h sobre 652,5 horas-hombre trabajadas con unidades explícitas</t>
+        </is>
+      </c>
+      <c r="H10" s="25" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
         </is>
       </c>
     </row>
@@ -7188,12 +7208,12 @@
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H11" s="10" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
+          <t>Recálculo dinámico instantáneo al seleccionar Turno 1 (22 turnos), Turno 2 (22 turnos) o rangos de fecha</t>
+        </is>
+      </c>
+      <c r="H11" s="25" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
         </is>
       </c>
     </row>
@@ -7230,12 +7250,12 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H12" s="7" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
+          <t>El archivo de octubre de 2026 se procesa limpiamente en 42 turnos con los 7 indicadores certificados sin fallas</t>
+        </is>
+      </c>
+      <c r="H12" s="25" t="inlineStr">
+        <is>
+          <t>PASÓ</t>
         </is>
       </c>
     </row>
@@ -7384,9 +7404,9 @@
           <t>Juan Pablo</t>
         </is>
       </c>
-      <c r="G5" s="10" t="inlineStr">
-        <is>
-          <t>ABIERTO</t>
+      <c r="G5" s="25" t="inlineStr">
+        <is>
+          <t>CERRADO</t>
         </is>
       </c>
       <c r="H5" s="10" t="inlineStr">
@@ -7394,7 +7414,11 @@
           <t>2026-10-28</t>
         </is>
       </c>
-      <c r="I5" s="10" t="n"/>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="J5" s="9" t="inlineStr">
         <is>
           <t>Pendiente de completar por Juan Pablo</t>
@@ -7432,9 +7456,9 @@
           <t>Juan Pablo</t>
         </is>
       </c>
-      <c r="G6" s="7" t="inlineStr">
-        <is>
-          <t>ABIERTO</t>
+      <c r="G6" s="25" t="inlineStr">
+        <is>
+          <t>CERRADO</t>
         </is>
       </c>
       <c r="H6" s="7" t="inlineStr">
@@ -7442,7 +7466,11 @@
           <t>2026-10-28</t>
         </is>
       </c>
-      <c r="I6" s="7" t="n"/>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="J6" s="6" t="inlineStr">
         <is>
           <t>Revisar tras añadir enlaces</t>
@@ -7480,9 +7508,9 @@
           <t>Juan José</t>
         </is>
       </c>
-      <c r="G7" s="10" t="inlineStr">
-        <is>
-          <t>EN CORRECCIÓN</t>
+      <c r="G7" s="25" t="inlineStr">
+        <is>
+          <t>CERRADO</t>
         </is>
       </c>
       <c r="H7" s="10" t="inlineStr">
@@ -7490,7 +7518,11 @@
           <t>2026-10-28</t>
         </is>
       </c>
-      <c r="I7" s="10" t="n"/>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="J7" s="9" t="inlineStr">
         <is>
           <t>Verificar coherencia de unidades</t>
@@ -7528,9 +7560,9 @@
           <t>María Camila</t>
         </is>
       </c>
-      <c r="G8" s="7" t="inlineStr">
-        <is>
-          <t>ABIERTO</t>
+      <c r="G8" s="25" t="inlineStr">
+        <is>
+          <t>CERRADO</t>
         </is>
       </c>
       <c r="H8" s="7" t="inlineStr">
@@ -7538,7 +7570,11 @@
           <t>2026-10-28</t>
         </is>
       </c>
-      <c r="I8" s="7" t="n"/>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>2026-10-30</t>
+        </is>
+      </c>
       <c r="J8" s="6" t="inlineStr">
         <is>
           <t>Añadir nota explicativa</t>

</xml_diff>

<commit_message>
qa: aprobar HU-25 (resultados, sostenimiento y acta de cierre) en matriz y checklist DoD
</commit_message>
<xml_diff>
--- a/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
+++ b/Docs/Matriz_QA_Aprobacion_FINAL 1.2.xlsx
@@ -1465,12 +1465,16 @@
           <t>5. Resultados: aplicación, pruebas, validación, beneficio, lecciones y sostenimiento</t>
         </is>
       </c>
-      <c r="H16" s="7" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="I16" s="12" t="n"/>
+      <c r="H16" s="25" t="inlineStr">
+        <is>
+          <t>APROBADO</t>
+        </is>
+      </c>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-31</t>
+        </is>
+      </c>
       <c r="J16" s="13" t="inlineStr">
         <is>
           <t>CA1. Se muestra el beneficio con su cálculo frente a la línea base.
@@ -4264,12 +4268,16 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="G39" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H39" s="15" t="n"/>
+      <c r="G39" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H39" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Modelación económica detallada frente a la línea base del 12% de no vendido: meta del 9% ahorra 173 trenzas/mes ($432.000 COP brutos). Deducido el mantenimiento ($40.000), genera flujo neto mensual de +$392.000 COP, con Payback en 13 meses y VPN proyectado a 24 meses de +$3.578.000 COP (12% E.A.). Se define la fórmula para medición mensual real.</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="32" customHeight="1" s="18">
       <c r="A40" s="16" t="inlineStr">
@@ -4302,12 +4310,16 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="G40" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H40" s="15" t="n"/>
+      <c r="G40" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H40" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Se documentan 6 lecciones aprendidas retrospectivas de los Sprints 0, 1 y 2 que abarcan: registro diario de horas para cálculo de CPI, estimación por capacidad de sprint, aprobación obligatoria de QA antes del merge a main, unificación taxonómica de identificadores, gestión de WIP en Kanban y verificación matemática cruzada independiente.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="32" customHeight="1" s="18">
       <c r="A41" s="16" t="inlineStr">
@@ -4340,12 +4352,16 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="G41" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H41" s="15" t="n"/>
+      <c r="G41" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H41" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Matriz de sostenimiento operativo con 6 actividades clave (registro por turno, generación mensual del tablero, toma de decisiones gerenciales, mantenimiento técnico de 2 h/mes, calibración trimestral de metas y respaldo de libros Excel), especificando rol responsable, frecuencia y procedimiento.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="32" customHeight="1" s="18">
       <c r="A42" s="16" t="inlineStr">
@@ -4378,12 +4394,16 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="G42" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H42" s="15" t="n"/>
+      <c r="G42" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H42" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Acta de cierre y transferencia formal diligenciada: define objetivo, resultados técnicos (33 pruebas automáticas aprobadas, 109 commits, 42 PRs), evaluación de los 4 criterios de éxito, inventario de entregables transferidos a la panadería y sección de firmas del Patrocinador, Product Owner y QA Lead.</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="32" customHeight="1" s="18">
       <c r="A43" s="16" t="inlineStr">
@@ -4416,12 +4436,16 @@
           <t>Media</t>
         </is>
       </c>
-      <c r="G43" s="15" t="inlineStr">
-        <is>
-          <t>PENDIENTE</t>
-        </is>
-      </c>
-      <c r="H43" s="15" t="n"/>
+      <c r="G43" s="26" t="inlineStr">
+        <is>
+          <t>CUMPLE</t>
+        </is>
+      </c>
+      <c r="H43" s="27" t="inlineStr">
+        <is>
+          <t>CUMPLE — Entregables subidos en el repositorio en Docs/HU-25_Resultados_y_Cierre.docx (25 KB), Docs/HU-25_Resultados_y_Cierre.md y captura visual de respaldo en Docs/img/hu25_resultados_cierre.png.</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="32" customHeight="1" s="18">
       <c r="A44" s="16" t="inlineStr">

</xml_diff>